<commit_message>
agregar kataleia diferentes detalles fase de finalizacion
</commit_message>
<xml_diff>
--- a/public/docs/fase2/Fase2-SprintBacklogAjuptel.xlsx
+++ b/public/docs/fase2/Fase2-SprintBacklogAjuptel.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="8"/>
   </bookViews>
   <sheets>
     <sheet name="Introducción" sheetId="1" state="visible" r:id="rId3"/>
@@ -4685,7 +4685,7 @@
       <c r="D31" s="63"/>
       <c r="XEO31" s="40"/>
     </row>
-    <row r="32" s="39" customFormat="true" ht="75.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="32" s="39" customFormat="true" ht="86.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B32" s="63" t="s">
         <v>100</v>
       </c>

</xml_diff>